<commit_message>
Agrupando la fecha de compra por mes y contando el numero de ventas hecha por cada uno, tambien hice el diagrama de lineas
</commit_message>
<xml_diff>
--- a/Data/Pen Sales Data Modificado 1er Ejercicio.xlsx
+++ b/Data/Pen Sales Data Modificado 1er Ejercicio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unanmanagua-my.sharepoint.com/personal/rene_sandoval23908226_estu_unan_edu_ni/Documents/UNAN 2023-2027/V Semestre/Analisis exploratorio de datos/Python 2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{CF10E04D-C46A-CB42-950C-0B504C1B54A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E77A194-BB36-465F-AA3A-CA3AD1B79739}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{CF10E04D-C46A-CB42-950C-0B504C1B54A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ED07ADC-A6CD-48CD-98CE-EAF4D73FC2E8}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19406" windowHeight="11486" xr2:uid="{88CB5200-0D19-2446-86AC-C4FBD1C615F9}"/>
   </bookViews>
@@ -240,6 +240,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -589,7 +593,7 @@
         <v>2.99</v>
       </c>
       <c r="E2" s="3">
-        <v>45047</v>
+        <v>44929</v>
       </c>
       <c r="F2" s="3">
         <v>44929</v>
@@ -613,7 +617,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3">
-        <v>45047</v>
+        <v>44930</v>
       </c>
       <c r="F3" s="3">
         <v>44930</v>
@@ -637,7 +641,7 @@
         <v>4.99</v>
       </c>
       <c r="E4" s="3">
-        <v>45047</v>
+        <v>44928</v>
       </c>
       <c r="F4" s="3">
         <v>44928</v>
@@ -661,7 +665,7 @@
         <v>2.99</v>
       </c>
       <c r="E5" s="3">
-        <v>45047</v>
+        <v>44961</v>
       </c>
       <c r="F5" s="3">
         <v>44961</v>
@@ -685,7 +689,7 @@
         <v>1.99</v>
       </c>
       <c r="E6" s="3">
-        <v>45047</v>
+        <v>44960</v>
       </c>
       <c r="F6" s="3">
         <v>44960</v>
@@ -709,7 +713,7 @@
         <v>1.99</v>
       </c>
       <c r="E7" s="3">
-        <v>45047</v>
+        <v>44961</v>
       </c>
       <c r="F7" s="3">
         <v>44961</v>
@@ -733,7 +737,7 @@
         <v>1.99</v>
       </c>
       <c r="E8" s="3">
-        <v>45047</v>
+        <v>44960</v>
       </c>
       <c r="F8" s="3">
         <v>44960</v>
@@ -757,7 +761,7 @@
         <v>1.99</v>
       </c>
       <c r="E9" s="3">
-        <v>45047</v>
+        <v>44964</v>
       </c>
       <c r="F9" s="3">
         <v>44964</v>
@@ -781,7 +785,7 @@
         <v>2.99</v>
       </c>
       <c r="E10" s="3">
-        <v>45047</v>
+        <v>44991</v>
       </c>
       <c r="F10" s="3">
         <v>44991</v>
@@ -805,7 +809,7 @@
         <v>4.99</v>
       </c>
       <c r="E11" s="3">
-        <v>45047</v>
+        <v>44987</v>
       </c>
       <c r="F11" s="3">
         <v>44987</v>
@@ -829,7 +833,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>45047</v>
+        <v>44989</v>
       </c>
       <c r="F12" s="3">
         <v>44989</v>
@@ -853,7 +857,7 @@
         <v>2.99</v>
       </c>
       <c r="E13" s="3">
-        <v>45047</v>
+        <v>45023</v>
       </c>
       <c r="F13" s="3">
         <v>45023</v>
@@ -877,7 +881,7 @@
         <v>1.99</v>
       </c>
       <c r="E14" s="3">
-        <v>45047</v>
+        <v>45019</v>
       </c>
       <c r="F14" s="3">
         <v>45019</v>
@@ -901,7 +905,7 @@
         <v>1.99</v>
       </c>
       <c r="E15" s="3">
-        <v>45047</v>
+        <v>45023</v>
       </c>
       <c r="F15" s="3">
         <v>45023</v>
@@ -924,8 +928,8 @@
       <c r="D16" s="2">
         <v>1.99</v>
       </c>
-      <c r="E16" s="3">
-        <v>45047</v>
+      <c r="E16" s="4">
+        <v>45019</v>
       </c>
       <c r="F16" s="4">
         <v>45019</v>
@@ -949,7 +953,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="3">
-        <v>45048</v>
+        <v>45020</v>
       </c>
       <c r="F17" s="3">
         <v>45020</v>
@@ -973,7 +977,7 @@
         <v>2.99</v>
       </c>
       <c r="E18" s="3">
-        <v>45048</v>
+        <v>45022</v>
       </c>
       <c r="F18" s="3">
         <v>45022</v>
@@ -996,8 +1000,8 @@
       <c r="D19" s="2">
         <v>4.99</v>
       </c>
-      <c r="E19" s="3">
-        <v>45048</v>
+      <c r="E19" s="4">
+        <v>45049</v>
       </c>
       <c r="F19" s="4">
         <v>45049</v>
@@ -1021,7 +1025,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="3">
-        <v>45048</v>
+        <v>45053</v>
       </c>
       <c r="F20" s="3">
         <v>45053</v>
@@ -1045,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="3">
-        <v>45048</v>
+        <v>45053</v>
       </c>
       <c r="F21" s="3">
         <v>45053</v>
@@ -1068,8 +1072,8 @@
       <c r="D22" s="2">
         <v>1.99</v>
       </c>
-      <c r="E22" s="3">
-        <v>45048</v>
+      <c r="E22" s="4">
+        <v>45051</v>
       </c>
       <c r="F22" s="4">
         <v>45051</v>
@@ -1092,8 +1096,8 @@
       <c r="D23" s="2">
         <v>1.99</v>
       </c>
-      <c r="E23" s="3">
-        <v>45048</v>
+      <c r="E23" s="4">
+        <v>45051</v>
       </c>
       <c r="F23" s="4">
         <v>45051</v>
@@ -1117,7 +1121,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="3">
-        <v>45048</v>
+        <v>45052</v>
       </c>
       <c r="F24" s="3">
         <v>45052</v>
@@ -1141,7 +1145,7 @@
         <v>2.99</v>
       </c>
       <c r="E25" s="3">
-        <v>45048</v>
+        <v>45052</v>
       </c>
       <c r="F25" s="3">
         <v>45052</v>
@@ -1165,7 +1169,7 @@
         <v>2.99</v>
       </c>
       <c r="E26" s="3">
-        <v>45048</v>
+        <v>45053</v>
       </c>
       <c r="F26" s="3">
         <v>45053</v>
@@ -1189,7 +1193,7 @@
         <v>1.99</v>
       </c>
       <c r="E27" s="3">
-        <v>45047</v>
+        <v>45080</v>
       </c>
       <c r="F27" s="3">
         <v>45080</v>
@@ -1211,7 +1215,7 @@
         <v>1.99</v>
       </c>
       <c r="E28" s="3">
-        <v>45047</v>
+        <v>45084</v>
       </c>
       <c r="F28" s="3">
         <v>45084</v>
@@ -1232,8 +1236,8 @@
       <c r="D29" s="2">
         <v>1.99</v>
       </c>
-      <c r="E29" s="3">
-        <v>45047</v>
+      <c r="E29" s="4">
+        <v>45080</v>
       </c>
       <c r="F29" s="4">
         <v>45080</v>
@@ -1255,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="3">
-        <v>45048</v>
+        <v>45111</v>
       </c>
       <c r="F30" s="3">
         <v>45111</v>
@@ -1277,7 +1281,7 @@
         <v>2.99</v>
       </c>
       <c r="E31" s="3">
-        <v>45048</v>
+        <v>45111</v>
       </c>
       <c r="F31" s="3">
         <v>45111</v>
@@ -1298,8 +1302,8 @@
       <c r="D32" s="2">
         <v>4.99</v>
       </c>
-      <c r="E32" s="3">
-        <v>45048</v>
+      <c r="E32" s="4">
+        <v>45110</v>
       </c>
       <c r="F32" s="4">
         <v>45110</v>
@@ -1321,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="3">
-        <v>45048</v>
+        <v>45145</v>
       </c>
       <c r="F33" s="3">
         <v>45145</v>
@@ -1343,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="3">
-        <v>45048</v>
+        <v>45145</v>
       </c>
       <c r="F34" s="3">
         <v>45145</v>
@@ -1364,8 +1368,8 @@
       <c r="D35" s="2">
         <v>1.99</v>
       </c>
-      <c r="E35" s="3">
-        <v>45048</v>
+      <c r="E35" s="4">
+        <v>45143</v>
       </c>
       <c r="F35" s="4">
         <v>45143</v>
@@ -1386,8 +1390,8 @@
       <c r="D36" s="2">
         <v>1.99</v>
       </c>
-      <c r="E36" s="3">
-        <v>45048</v>
+      <c r="E36" s="4">
+        <v>45143</v>
       </c>
       <c r="F36" s="4">
         <v>45143</v>
@@ -1409,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="E37" s="3">
-        <v>45048</v>
+        <v>45175</v>
       </c>
       <c r="F37" s="3">
         <v>45175</v>
@@ -1431,7 +1435,7 @@
         <v>2.99</v>
       </c>
       <c r="E38" s="3">
-        <v>45048</v>
+        <v>45175</v>
       </c>
       <c r="F38" s="3">
         <v>45175</v>
@@ -1453,7 +1457,7 @@
         <v>2.99</v>
       </c>
       <c r="E39" s="3">
-        <v>45048</v>
+        <v>45176</v>
       </c>
       <c r="F39" s="3">
         <v>45176</v>
@@ -1536,21 +1540,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AD83AFDB133AE84091E51804354FA7EE" ma:contentTypeVersion="8" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="f49275ace62bf5fa599342d318323630">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bb583d6-7de5-4467-bb06-9aeb8738f185" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0d007ce636fb2ce637e66dc94a6f9197" ns2:_="">
     <xsd:import namespace="1bb583d6-7de5-4467-bb06-9aeb8738f185"/>
@@ -1718,24 +1707,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DF9CF85-D68B-497D-B89F-259FC52725F2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7F82D2F-E708-4223-A587-34EE88DDC2ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD506EFA-CF68-4EB5-A8AA-F6E42D705E41}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1751,4 +1738,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7F82D2F-E708-4223-A587-34EE88DDC2ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DF9CF85-D68B-497D-B89F-259FC52725F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>